<commit_message>
add German column headers
</commit_message>
<xml_diff>
--- a/static/excel/pool-importvorlage-minimal.xlsx
+++ b/static/excel/pool-importvorlage-minimal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgr/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1707732B-2B65-454A-BAFA-0F21C5612DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860E68CC-CA9B-9542-B56F-079BDA87D571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="54160" yWindow="600" windowWidth="34140" windowHeight="19440" xr2:uid="{D7DA82DE-661B-4434-8FCB-AD97B6E46B4F}"/>
   </bookViews>
@@ -38,48 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
-    <t>number</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>longDescription</t>
-  </si>
-  <si>
-    <t>orderUnit</t>
-  </si>
-  <si>
-    <t>contentUnit</t>
-  </si>
-  <si>
-    <t>contentQuantity</t>
-  </si>
-  <si>
-    <t>minimumOrderQuantity</t>
-  </si>
-  <si>
-    <t>price1</t>
-  </si>
-  <si>
-    <t>quantity1</t>
-  </si>
-  <si>
-    <t>price3</t>
-  </si>
-  <si>
-    <t>price2</t>
-  </si>
-  <si>
-    <t>quantity2</t>
-  </si>
-  <si>
-    <t>quantity3</t>
-  </si>
-  <si>
-    <t>files1</t>
-  </si>
-  <si>
     <t>12345-001</t>
   </si>
   <si>
@@ -96,6 +54,48 @@
   </si>
   <si>
     <t>http(s)://example.com/bilder/artikelbild1.jpg</t>
+  </si>
+  <si>
+    <t>number (Artikelnummer)</t>
+  </si>
+  <si>
+    <t>name (Artikelname)</t>
+  </si>
+  <si>
+    <t>longDescription (Artikelbeschreibung)</t>
+  </si>
+  <si>
+    <t>orderUnit (Bestelleinheit)</t>
+  </si>
+  <si>
+    <t>contentUnit (Inhaltseinheit)</t>
+  </si>
+  <si>
+    <t>contentQuantity (Inhaltsmenge)</t>
+  </si>
+  <si>
+    <t>minimumOrderQuantity (Mindestbestellmenge)</t>
+  </si>
+  <si>
+    <t>price1 (Preis1)</t>
+  </si>
+  <si>
+    <t>quantity1 (Preis1 - ab Menge)</t>
+  </si>
+  <si>
+    <t>quantity2 (Preis2- ab Menge)</t>
+  </si>
+  <si>
+    <t>quantity3 (Preis3 - ab Menge)</t>
+  </si>
+  <si>
+    <t>price2 (Preis2)</t>
+  </si>
+  <si>
+    <t>price3 (Preis3)</t>
+  </si>
+  <si>
+    <t>files1 (Artikelbild)</t>
   </si>
 </sst>
 </file>
@@ -465,69 +465,81 @@
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="22.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="36.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="F2">
         <v>25</v>
@@ -554,7 +566,7 @@
         <v>15</v>
       </c>
       <c r="N2" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -836,9 +848,31 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3718C1D1-56D9-4D62-B988-9AC37FE60611}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3718C1D1-56D9-4D62-B988-9AC37FE60611}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="972a4302-61b6-4e60-8451-b9c9ef50fbef"/>
+    <ds:schemaRef ds:uri="c9de2a3f-a2ad-4682-ba79-07e79da285ff"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10B9212C-C94A-4C34-8339-5A6F865954FA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10B9212C-C94A-4C34-8339-5A6F865954FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c9de2a3f-a2ad-4682-ba79-07e79da285ff"/>
+    <ds:schemaRef ds:uri="972a4302-61b6-4e60-8451-b9c9ef50fbef"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>